<commit_message>
"mobile progress bar fit and stat update"
</commit_message>
<xml_diff>
--- a/site/statindexs/Ratings.xlsx
+++ b/site/statindexs/Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nathaniel\Documents\GitHub\ppro\site\statindexs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{710542D0-1921-46FF-BF48-B305EFE84BF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22946800-11B3-4135-828C-C11BE574AE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4245" yWindow="1815" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2105" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2098" uniqueCount="165">
   <si>
     <t>Fighter Name</t>
   </si>
@@ -609,7 +609,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FighterStatsTable" displayName="FighterStatsTable" ref="A1:H139" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="FighterStatsTable" displayName="FighterStatsTable" ref="A1:H132" totalsRowShown="0">
   <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Fighter Name"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="CHIN"/>
@@ -830,7 +830,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H139"/>
+  <dimension ref="A1:H132"/>
   <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
@@ -1619,311 +1619,311 @@
     </row>
     <row r="31" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A31" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B31" s="2">
-        <v>92</v>
+        <v>85</v>
       </c>
       <c r="C31" s="2">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D31" s="2">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E31" s="2">
+        <v>97</v>
+      </c>
+      <c r="F31" s="2">
         <v>91</v>
       </c>
-      <c r="F31" s="2">
-        <v>97</v>
-      </c>
       <c r="G31" s="2">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="H31" s="2">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A32" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B32" s="2">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C32" s="2">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="D32" s="2">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="E32" s="2">
+        <v>84</v>
+      </c>
+      <c r="F32" s="2">
+        <v>78</v>
+      </c>
+      <c r="G32" s="2">
+        <v>100</v>
+      </c>
+      <c r="H32" s="2">
         <v>97</v>
-      </c>
-      <c r="F32" s="2">
-        <v>91</v>
-      </c>
-      <c r="G32" s="2">
-        <v>91</v>
-      </c>
-      <c r="H32" s="2">
-        <v>90</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A33" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B33" s="2">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="C33" s="2">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D33" s="2">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="E33" s="2">
+        <v>97</v>
+      </c>
+      <c r="F33" s="2">
+        <v>92</v>
+      </c>
+      <c r="G33" s="2">
         <v>91</v>
       </c>
-      <c r="F33" s="2">
-        <v>93</v>
-      </c>
-      <c r="G33" s="2">
-        <v>90</v>
-      </c>
       <c r="H33" s="2">
-        <v>91</v>
+        <v>86</v>
       </c>
     </row>
     <row r="34" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A34" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B34" s="2">
+        <v>89</v>
+      </c>
+      <c r="C34" s="2">
+        <v>92</v>
+      </c>
+      <c r="D34" s="2">
         <v>87</v>
       </c>
-      <c r="C34" s="2">
-        <v>86</v>
-      </c>
-      <c r="D34" s="2">
+      <c r="E34" s="2">
         <v>90</v>
       </c>
-      <c r="E34" s="2">
-        <v>84</v>
-      </c>
       <c r="F34" s="2">
-        <v>78</v>
+        <v>90</v>
       </c>
       <c r="G34" s="2">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H34" s="2">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
     <row r="35" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A35" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B35" s="2">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="C35" s="2">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="D35" s="2">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="E35" s="2">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="F35" s="2">
+        <v>72</v>
+      </c>
+      <c r="G35" s="2">
         <v>92</v>
       </c>
-      <c r="G35" s="2">
-        <v>91</v>
-      </c>
       <c r="H35" s="2">
-        <v>86</v>
+        <v>78</v>
       </c>
     </row>
     <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A36" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B36" s="2">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C36" s="2">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="D36" s="2">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="E36" s="2">
         <v>90</v>
       </c>
       <c r="F36" s="2">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G36" s="2">
-        <v>99</v>
+        <v>70</v>
       </c>
       <c r="H36" s="2">
-        <v>99</v>
+        <v>72</v>
       </c>
     </row>
     <row r="37" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A37" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B37" s="2">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C37" s="2">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="D37" s="2">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E37" s="2">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="F37" s="2">
+        <v>80</v>
+      </c>
+      <c r="G37" s="2">
+        <v>84</v>
+      </c>
+      <c r="H37" s="2">
         <v>82</v>
-      </c>
-      <c r="G37" s="2">
-        <v>78</v>
-      </c>
-      <c r="H37" s="2">
-        <v>92</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A38" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B38" s="2">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C38" s="2">
+        <v>96</v>
+      </c>
+      <c r="D38" s="2">
+        <v>79</v>
+      </c>
+      <c r="E38" s="2">
+        <v>93</v>
+      </c>
+      <c r="F38" s="2">
+        <v>85</v>
+      </c>
+      <c r="G38" s="2">
         <v>94</v>
       </c>
-      <c r="D38" s="2">
-        <v>94</v>
-      </c>
-      <c r="E38" s="2">
-        <v>92</v>
-      </c>
-      <c r="F38" s="2">
-        <v>72</v>
-      </c>
-      <c r="G38" s="2">
-        <v>92</v>
-      </c>
       <c r="H38" s="2">
-        <v>78</v>
+        <v>84</v>
       </c>
     </row>
     <row r="39" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A39" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B39" s="2">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C39" s="2">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D39" s="2">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="E39" s="2">
-        <v>79</v>
+        <v>94</v>
       </c>
       <c r="F39" s="2">
-        <v>72</v>
+        <v>92</v>
       </c>
       <c r="G39" s="2">
-        <v>97</v>
+        <v>78</v>
       </c>
       <c r="H39" s="2">
-        <v>97</v>
+        <v>84</v>
       </c>
     </row>
     <row r="40" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A40" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B40" s="2">
+        <v>94</v>
+      </c>
+      <c r="C40" s="2">
+        <v>96</v>
+      </c>
+      <c r="D40" s="2">
+        <v>82</v>
+      </c>
+      <c r="E40" s="2">
         <v>88</v>
       </c>
-      <c r="C40" s="2">
-        <v>90</v>
-      </c>
-      <c r="D40" s="2">
-        <v>84</v>
-      </c>
-      <c r="E40" s="2">
-        <v>94</v>
-      </c>
       <c r="F40" s="2">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="G40" s="2">
         <v>86</v>
       </c>
       <c r="H40" s="2">
-        <v>92</v>
+        <v>95</v>
       </c>
     </row>
     <row r="41" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A41" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B41" s="2">
+        <v>92</v>
+      </c>
+      <c r="C41" s="2">
+        <v>99</v>
+      </c>
+      <c r="D41" s="2">
         <v>82</v>
       </c>
-      <c r="C41" s="2">
-        <v>83</v>
-      </c>
-      <c r="D41" s="2">
-        <v>95</v>
-      </c>
       <c r="E41" s="2">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="F41" s="2">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="G41" s="2">
-        <v>70</v>
+        <v>96</v>
       </c>
       <c r="H41" s="2">
-        <v>72</v>
+        <v>98</v>
       </c>
     </row>
     <row r="42" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A42" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B42" s="2">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C42" s="2">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D42" s="2">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="E42" s="2">
-        <v>93</v>
+        <v>85</v>
       </c>
       <c r="F42" s="2">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="G42" s="2">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="H42" s="2">
         <v>82</v>
@@ -1931,519 +1931,519 @@
     </row>
     <row r="43" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A43" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B43" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C43" s="2">
+        <v>83</v>
+      </c>
+      <c r="D43" s="2">
         <v>96</v>
       </c>
-      <c r="D43" s="2">
+      <c r="E43" s="2">
+        <v>94</v>
+      </c>
+      <c r="F43" s="2">
+        <v>97</v>
+      </c>
+      <c r="G43" s="2">
         <v>79</v>
       </c>
-      <c r="E43" s="2">
-        <v>93</v>
-      </c>
-      <c r="F43" s="2">
-        <v>85</v>
-      </c>
-      <c r="G43" s="2">
-        <v>94</v>
-      </c>
       <c r="H43" s="2">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="44" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A44" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B44" s="2">
+        <v>90</v>
+      </c>
+      <c r="C44" s="2">
+        <v>95</v>
+      </c>
+      <c r="D44" s="2">
+        <v>87</v>
+      </c>
+      <c r="E44" s="2">
         <v>89</v>
       </c>
-      <c r="C44" s="2">
+      <c r="F44" s="2">
+        <v>94</v>
+      </c>
+      <c r="G44" s="2">
         <v>87</v>
       </c>
-      <c r="D44" s="2">
-        <v>96</v>
-      </c>
-      <c r="E44" s="2">
-        <v>94</v>
-      </c>
-      <c r="F44" s="2">
-        <v>92</v>
-      </c>
-      <c r="G44" s="2">
-        <v>78</v>
-      </c>
       <c r="H44" s="2">
-        <v>84</v>
+        <v>93</v>
       </c>
     </row>
     <row r="45" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A45" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B45" s="2">
-        <v>94</v>
+        <v>84</v>
       </c>
       <c r="C45" s="2">
+        <v>97</v>
+      </c>
+      <c r="D45" s="2">
+        <v>90</v>
+      </c>
+      <c r="E45" s="2">
         <v>96</v>
       </c>
-      <c r="D45" s="2">
-        <v>82</v>
-      </c>
-      <c r="E45" s="2">
+      <c r="F45" s="2">
+        <v>93</v>
+      </c>
+      <c r="G45" s="2">
+        <v>92</v>
+      </c>
+      <c r="H45" s="2">
         <v>88</v>
-      </c>
-      <c r="F45" s="2">
-        <v>87</v>
-      </c>
-      <c r="G45" s="2">
-        <v>86</v>
-      </c>
-      <c r="H45" s="2">
-        <v>95</v>
       </c>
     </row>
     <row r="46" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A46" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B46" s="2">
+        <v>88</v>
+      </c>
+      <c r="C46" s="2">
+        <v>81</v>
+      </c>
+      <c r="D46" s="2">
+        <v>99</v>
+      </c>
+      <c r="E46" s="2">
         <v>92</v>
       </c>
-      <c r="C46" s="2">
-        <v>99</v>
-      </c>
-      <c r="D46" s="2">
-        <v>82</v>
-      </c>
-      <c r="E46" s="2">
-        <v>97</v>
-      </c>
       <c r="F46" s="2">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="G46" s="2">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="H46" s="2">
-        <v>98</v>
+        <v>92</v>
       </c>
     </row>
     <row r="47" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A47" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B47" s="2">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C47" s="2">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="D47" s="2">
-        <v>76</v>
+        <v>92</v>
       </c>
       <c r="E47" s="2">
-        <v>85</v>
+        <v>94</v>
       </c>
       <c r="F47" s="2">
-        <v>83</v>
+        <v>98</v>
       </c>
       <c r="G47" s="2">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="H47" s="2">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A48" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B48" s="2">
-        <v>83</v>
+        <v>95</v>
       </c>
       <c r="C48" s="2">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="D48" s="2">
-        <v>96</v>
+        <v>92</v>
       </c>
       <c r="E48" s="2">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F48" s="2">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="G48" s="2">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="H48" s="2">
-        <v>74</v>
+        <v>95</v>
       </c>
     </row>
     <row r="49" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A49" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B49" s="2">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C49" s="2">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="D49" s="2">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="E49" s="2">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F49" s="2">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="G49" s="2">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H49" s="2">
-        <v>93</v>
+        <v>98</v>
       </c>
     </row>
     <row r="50" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A50" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B50" s="2">
+        <v>94</v>
+      </c>
+      <c r="C50" s="2">
+        <v>98</v>
+      </c>
+      <c r="D50" s="2">
         <v>84</v>
-      </c>
-      <c r="C50" s="2">
-        <v>97</v>
-      </c>
-      <c r="D50" s="2">
-        <v>90</v>
       </c>
       <c r="E50" s="2">
         <v>96</v>
       </c>
       <c r="F50" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="G50" s="2">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="H50" s="2">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="51" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A51" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B51" s="2">
+        <v>91</v>
+      </c>
+      <c r="C51" s="2">
+        <v>96</v>
+      </c>
+      <c r="D51" s="2">
+        <v>92</v>
+      </c>
+      <c r="E51" s="2">
         <v>88</v>
       </c>
-      <c r="C51" s="2">
-        <v>81</v>
-      </c>
-      <c r="D51" s="2">
-        <v>99</v>
-      </c>
-      <c r="E51" s="2">
-        <v>92</v>
-      </c>
       <c r="F51" s="2">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="G51" s="2">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="H51" s="2">
-        <v>92</v>
+        <v>84</v>
       </c>
     </row>
     <row r="52" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A52" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B52" s="2">
         <v>89</v>
       </c>
       <c r="C52" s="2">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D52" s="2">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="E52" s="2">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="F52" s="2">
-        <v>98</v>
+        <v>68</v>
       </c>
       <c r="G52" s="2">
-        <v>69</v>
+        <v>96</v>
       </c>
       <c r="H52" s="2">
-        <v>80</v>
+        <v>89</v>
       </c>
     </row>
     <row r="53" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A53" t="s">
-        <v>59</v>
+        <v>66</v>
       </c>
       <c r="B53" s="2">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C53" s="2">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D53" s="2">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="E53" s="2">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="F53" s="2">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G53" s="2">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="H53" s="2">
-        <v>95</v>
+        <v>99</v>
       </c>
     </row>
     <row r="54" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A54" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="B54" s="2">
+        <v>89</v>
+      </c>
+      <c r="C54" s="2">
         <v>93</v>
       </c>
-      <c r="C54" s="2">
+      <c r="D54" s="2">
+        <v>82</v>
+      </c>
+      <c r="E54" s="2">
+        <v>90</v>
+      </c>
+      <c r="F54" s="2">
+        <v>89</v>
+      </c>
+      <c r="G54" s="2">
+        <v>90</v>
+      </c>
+      <c r="H54" s="2">
         <v>92</v>
-      </c>
-      <c r="D54" s="2">
-        <v>91</v>
-      </c>
-      <c r="E54" s="2">
-        <v>91</v>
-      </c>
-      <c r="F54" s="2">
-        <v>91</v>
-      </c>
-      <c r="G54" s="2">
-        <v>93</v>
-      </c>
-      <c r="H54" s="2">
-        <v>98</v>
       </c>
     </row>
     <row r="55" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A55" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="B55" s="2">
         <v>94</v>
       </c>
       <c r="C55" s="2">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="D55" s="2">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="E55" s="2">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="F55" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="G55" s="2">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H55" s="2">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="56" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A56" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="B56" s="2">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C56" s="2">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="D56" s="2">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="E56" s="2">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F56" s="2">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="G56" s="2">
-        <v>98</v>
+        <v>78</v>
       </c>
       <c r="H56" s="2">
-        <v>84</v>
+        <v>99</v>
       </c>
     </row>
     <row r="57" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A57" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="B57" s="2">
-        <v>89</v>
+        <v>68</v>
       </c>
       <c r="C57" s="2">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="D57" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="E57" s="2">
+        <v>94</v>
+      </c>
+      <c r="F57" s="2">
+        <v>86</v>
+      </c>
+      <c r="G57" s="2">
+        <v>88</v>
+      </c>
+      <c r="H57" s="2">
         <v>78</v>
-      </c>
-      <c r="F57" s="2">
-        <v>68</v>
-      </c>
-      <c r="G57" s="2">
-        <v>96</v>
-      </c>
-      <c r="H57" s="2">
-        <v>89</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A58" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="B58" s="2">
-        <v>80</v>
+        <v>92</v>
       </c>
       <c r="C58" s="2">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="D58" s="2">
-        <v>84</v>
+        <v>94</v>
       </c>
       <c r="E58" s="2">
-        <v>72</v>
+        <v>91</v>
       </c>
       <c r="F58" s="2">
-        <v>60</v>
+        <v>89</v>
       </c>
       <c r="G58" s="2">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="H58" s="2">
-        <v>99</v>
+        <v>96</v>
       </c>
     </row>
     <row r="59" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A59" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="B59" s="2">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="C59" s="2">
+        <v>91</v>
+      </c>
+      <c r="D59" s="2">
+        <v>85</v>
+      </c>
+      <c r="E59" s="2">
         <v>89</v>
       </c>
-      <c r="D59" s="2">
-        <v>99</v>
-      </c>
-      <c r="E59" s="2">
+      <c r="F59" s="2">
         <v>94</v>
       </c>
-      <c r="F59" s="2">
-        <v>92</v>
-      </c>
       <c r="G59" s="2">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H59" s="2">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="60" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A60" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="B60" s="2">
-        <v>96</v>
+        <v>85</v>
       </c>
       <c r="C60" s="2">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D60" s="2">
+        <v>78</v>
+      </c>
+      <c r="E60" s="2">
         <v>87</v>
       </c>
-      <c r="E60" s="2">
-        <v>88</v>
-      </c>
       <c r="F60" s="2">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="G60" s="2">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="H60" s="2">
-        <v>99</v>
+        <v>97</v>
       </c>
     </row>
     <row r="61" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A61" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="B61" s="2">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="C61" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D61" s="2">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="E61" s="2">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F61" s="2">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="G61" s="2">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="H61" s="2">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="62" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A62" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="B62" s="2">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="C62" s="2">
+        <v>97</v>
+      </c>
+      <c r="D62" s="2">
+        <v>86</v>
+      </c>
+      <c r="E62" s="2">
+        <v>97</v>
+      </c>
+      <c r="F62" s="2">
+        <v>96</v>
+      </c>
+      <c r="G62" s="2">
         <v>89</v>
-      </c>
-      <c r="D62" s="2">
-        <v>94</v>
-      </c>
-      <c r="E62" s="2">
-        <v>94</v>
-      </c>
-      <c r="F62" s="2">
-        <v>92</v>
-      </c>
-      <c r="G62" s="2">
-        <v>90</v>
       </c>
       <c r="H62" s="2">
         <v>87</v>
@@ -2451,374 +2451,374 @@
     </row>
     <row r="63" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A63" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="B63" s="2">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C63" s="2">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D63" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="E63" s="2">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F63" s="2">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="G63" s="2">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="H63" s="2">
-        <v>99</v>
+        <v>86</v>
       </c>
     </row>
     <row r="64" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A64" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="B64" s="2">
-        <v>68</v>
+        <v>89</v>
       </c>
       <c r="C64" s="2">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="D64" s="2">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="E64" s="2">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="F64" s="2">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="G64" s="2">
-        <v>88</v>
+        <v>76</v>
       </c>
       <c r="H64" s="2">
-        <v>78</v>
+        <v>96</v>
       </c>
     </row>
     <row r="65" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A65" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="B65" s="2">
+        <v>90</v>
+      </c>
+      <c r="C65" s="2">
+        <v>94</v>
+      </c>
+      <c r="D65" s="2">
         <v>92</v>
       </c>
-      <c r="C65" s="2">
-        <v>91</v>
-      </c>
-      <c r="D65" s="2">
-        <v>94</v>
-      </c>
       <c r="E65" s="2">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F65" s="2">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="G65" s="2">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="H65" s="2">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A66" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="B66" s="2">
+        <v>90</v>
+      </c>
+      <c r="C66" s="2">
+        <v>95</v>
+      </c>
+      <c r="D66" s="2">
+        <v>92</v>
+      </c>
+      <c r="E66" s="2">
+        <v>95</v>
+      </c>
+      <c r="F66" s="2">
+        <v>87</v>
+      </c>
+      <c r="G66" s="2">
         <v>86</v>
       </c>
-      <c r="C66" s="2">
-        <v>91</v>
-      </c>
-      <c r="D66" s="2">
-        <v>85</v>
-      </c>
-      <c r="E66" s="2">
+      <c r="H66" s="2">
         <v>89</v>
-      </c>
-      <c r="F66" s="2">
-        <v>94</v>
-      </c>
-      <c r="G66" s="2">
-        <v>96</v>
-      </c>
-      <c r="H66" s="2">
-        <v>96</v>
       </c>
     </row>
     <row r="67" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A67" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="B67" s="2">
+        <v>90</v>
+      </c>
+      <c r="C67" s="2">
+        <v>92</v>
+      </c>
+      <c r="D67" s="2">
         <v>85</v>
-      </c>
-      <c r="C67" s="2">
-        <v>95</v>
-      </c>
-      <c r="D67" s="2">
-        <v>78</v>
       </c>
       <c r="E67" s="2">
         <v>87</v>
       </c>
       <c r="F67" s="2">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G67" s="2">
-        <v>97</v>
+        <v>74</v>
       </c>
       <c r="H67" s="2">
-        <v>97</v>
+        <v>88</v>
       </c>
     </row>
     <row r="68" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A68" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="B68" s="2">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="C68" s="2">
+        <v>91</v>
+      </c>
+      <c r="D68" s="2">
         <v>92</v>
       </c>
-      <c r="D68" s="2">
-        <v>88</v>
-      </c>
       <c r="E68" s="2">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="F68" s="2">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="G68" s="2">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="H68" s="2">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="69" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A69" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B69" s="2">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C69" s="2">
-        <v>97</v>
+        <v>93</v>
       </c>
       <c r="D69" s="2">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E69" s="2">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="F69" s="2">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="G69" s="2">
         <v>89</v>
       </c>
       <c r="H69" s="2">
-        <v>87</v>
+        <v>84</v>
       </c>
     </row>
     <row r="70" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A70" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B70" s="2">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C70" s="2">
-        <v>95</v>
+        <v>88</v>
       </c>
       <c r="D70" s="2">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="E70" s="2">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F70" s="2">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G70" s="2">
-        <v>98</v>
+        <v>77</v>
       </c>
       <c r="H70" s="2">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="71" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A71" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="B71" s="2">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="C71" s="2">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="D71" s="2">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E71" s="2">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="F71" s="2">
         <v>89</v>
       </c>
       <c r="G71" s="2">
-        <v>76</v>
+        <v>94</v>
       </c>
       <c r="H71" s="2">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="72" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A72" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="B72" s="2">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C72" s="2">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D72" s="2">
-        <v>92</v>
+        <v>74</v>
       </c>
       <c r="E72" s="2">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F72" s="2">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="G72" s="2">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H72" s="2">
-        <v>95</v>
+        <v>91</v>
       </c>
     </row>
     <row r="73" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A73" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B73" s="2">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="C73" s="2">
+        <v>91</v>
+      </c>
+      <c r="D73" s="2">
+        <v>88</v>
+      </c>
+      <c r="E73" s="2">
+        <v>87</v>
+      </c>
+      <c r="F73" s="2">
+        <v>97</v>
+      </c>
+      <c r="G73" s="2">
+        <v>83</v>
+      </c>
+      <c r="H73" s="2">
         <v>95</v>
-      </c>
-      <c r="D73" s="2">
-        <v>92</v>
-      </c>
-      <c r="E73" s="2">
-        <v>95</v>
-      </c>
-      <c r="F73" s="2">
-        <v>87</v>
-      </c>
-      <c r="G73" s="2">
-        <v>86</v>
-      </c>
-      <c r="H73" s="2">
-        <v>89</v>
       </c>
     </row>
     <row r="74" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A74" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B74" s="2">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C74" s="2">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="D74" s="2">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="E74" s="2">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="F74" s="2">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="G74" s="2">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="H74" s="2">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="75" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A75" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="B75" s="2">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C75" s="2">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="D75" s="2">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="E75" s="2">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="F75" s="2">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="G75" s="2">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="H75" s="2">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="76" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A76" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B76" s="2">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="C76" s="2">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="D76" s="2">
+        <v>87</v>
+      </c>
+      <c r="E76" s="2">
         <v>88</v>
       </c>
-      <c r="E76" s="2">
-        <v>94</v>
-      </c>
       <c r="F76" s="2">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="G76" s="2">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="H76" s="2">
-        <v>84</v>
+        <v>96</v>
       </c>
     </row>
     <row r="77" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A77" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="B77" s="2">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="C77" s="2">
         <v>88</v>
@@ -2827,362 +2827,362 @@
         <v>96</v>
       </c>
       <c r="E77" s="2">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="F77" s="2">
         <v>93</v>
       </c>
       <c r="G77" s="2">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="H77" s="2">
-        <v>84</v>
+        <v>74</v>
       </c>
     </row>
     <row r="78" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A78" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B78" s="2">
         <v>83</v>
       </c>
       <c r="C78" s="2">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="D78" s="2">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="E78" s="2">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="F78" s="2">
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="G78" s="2">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="H78" s="2">
-        <v>95</v>
+        <v>84</v>
       </c>
     </row>
     <row r="79" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A79" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="B79" s="2">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="C79" s="2">
-        <v>95</v>
+        <v>87</v>
       </c>
       <c r="D79" s="2">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E79" s="2">
         <v>88</v>
       </c>
       <c r="F79" s="2">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G79" s="2">
-        <v>98</v>
+        <v>89</v>
       </c>
       <c r="H79" s="2">
-        <v>91</v>
+        <v>97</v>
       </c>
     </row>
     <row r="80" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A80" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B80" s="2">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C80" s="2">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D80" s="2">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="E80" s="2">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F80" s="2">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="G80" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="H80" s="2">
-        <v>95</v>
+        <v>92</v>
       </c>
     </row>
     <row r="81" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A81" t="s">
+        <v>94</v>
+      </c>
+      <c r="B81" s="2">
+        <v>92</v>
+      </c>
+      <c r="C81" s="2">
         <v>87</v>
       </c>
-      <c r="B81" s="2">
+      <c r="D81" s="2">
+        <v>93</v>
+      </c>
+      <c r="E81" s="2">
+        <v>92</v>
+      </c>
+      <c r="F81" s="2">
         <v>91</v>
       </c>
-      <c r="C81" s="2">
-        <v>99</v>
-      </c>
-      <c r="D81" s="2">
-        <v>83</v>
-      </c>
-      <c r="E81" s="2">
-        <v>91</v>
-      </c>
-      <c r="F81" s="2">
+      <c r="G81" s="2">
         <v>82</v>
       </c>
-      <c r="G81" s="2">
-        <v>96</v>
-      </c>
       <c r="H81" s="2">
-        <v>89</v>
+        <v>86</v>
       </c>
     </row>
     <row r="82" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A82" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B82" s="2">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C82" s="2">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="D82" s="2">
-        <v>97</v>
+        <v>87</v>
       </c>
       <c r="E82" s="2">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="F82" s="2">
-        <v>86</v>
+        <v>96</v>
       </c>
       <c r="G82" s="2">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="H82" s="2">
-        <v>88</v>
+        <v>84</v>
       </c>
     </row>
     <row r="83" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A83" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B83" s="2">
+        <v>91</v>
+      </c>
+      <c r="C83" s="2">
         <v>99</v>
-      </c>
-      <c r="C83" s="2">
-        <v>98</v>
       </c>
       <c r="D83" s="2">
         <v>87</v>
       </c>
       <c r="E83" s="2">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F83" s="2">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="G83" s="2">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="H83" s="2">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="84" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A84" t="s">
+        <v>97</v>
+      </c>
+      <c r="B84" s="2">
         <v>90</v>
       </c>
-      <c r="B84" s="2">
+      <c r="C84" s="2">
+        <v>92</v>
+      </c>
+      <c r="D84" s="2">
+        <v>89</v>
+      </c>
+      <c r="E84" s="2">
+        <v>91</v>
+      </c>
+      <c r="F84" s="2">
         <v>85</v>
       </c>
-      <c r="C84" s="2">
-        <v>88</v>
-      </c>
-      <c r="D84" s="2">
-        <v>96</v>
-      </c>
-      <c r="E84" s="2">
-        <v>88</v>
-      </c>
-      <c r="F84" s="2">
-        <v>93</v>
-      </c>
       <c r="G84" s="2">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="H84" s="2">
-        <v>74</v>
+        <v>82</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A85" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="B85" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C85" s="2">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="D85" s="2">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="E85" s="2">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F85" s="2">
-        <v>81</v>
+        <v>99</v>
       </c>
       <c r="G85" s="2">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="H85" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
     </row>
     <row r="86" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A86" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B86" s="2">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C86" s="2">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D86" s="2">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="E86" s="2">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F86" s="2">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="G86" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="H86" s="2">
-        <v>97</v>
+        <v>86</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A87" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="B87" s="2">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="C87" s="2">
+        <v>94</v>
+      </c>
+      <c r="D87" s="2">
+        <v>88</v>
+      </c>
+      <c r="E87" s="2">
+        <v>94</v>
+      </c>
+      <c r="F87" s="2">
         <v>95</v>
       </c>
-      <c r="D87" s="2">
-        <v>78</v>
-      </c>
-      <c r="E87" s="2">
-        <v>84</v>
-      </c>
-      <c r="F87" s="2">
-        <v>82</v>
-      </c>
       <c r="G87" s="2">
-        <v>96</v>
+        <v>86</v>
       </c>
       <c r="H87" s="2">
-        <v>92</v>
+        <v>85</v>
       </c>
     </row>
     <row r="88" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A88" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="B88" s="2">
-        <v>92</v>
+        <v>83</v>
       </c>
       <c r="C88" s="2">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="D88" s="2">
-        <v>93</v>
+        <v>80</v>
       </c>
       <c r="E88" s="2">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="F88" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="G88" s="2">
-        <v>82</v>
+        <v>96</v>
       </c>
       <c r="H88" s="2">
-        <v>86</v>
+        <v>98</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A89" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B89" s="2">
+        <v>88</v>
+      </c>
+      <c r="C89" s="2">
+        <v>86</v>
+      </c>
+      <c r="D89" s="2">
+        <v>92</v>
+      </c>
+      <c r="E89" s="2">
+        <v>84</v>
+      </c>
+      <c r="F89" s="2">
+        <v>80</v>
+      </c>
+      <c r="G89" s="2">
+        <v>99</v>
+      </c>
+      <c r="H89" s="2">
         <v>89</v>
-      </c>
-      <c r="C89" s="2">
-        <v>95</v>
-      </c>
-      <c r="D89" s="2">
-        <v>87</v>
-      </c>
-      <c r="E89" s="2">
-        <v>95</v>
-      </c>
-      <c r="F89" s="2">
-        <v>96</v>
-      </c>
-      <c r="G89" s="2">
-        <v>85</v>
-      </c>
-      <c r="H89" s="2">
-        <v>84</v>
       </c>
     </row>
     <row r="90" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A90" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="B90" s="2">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="C90" s="2">
-        <v>99</v>
+        <v>86</v>
       </c>
       <c r="D90" s="2">
+        <v>97</v>
+      </c>
+      <c r="E90" s="2">
         <v>87</v>
       </c>
-      <c r="E90" s="2">
-        <v>94</v>
-      </c>
       <c r="F90" s="2">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="G90" s="2">
-        <v>99</v>
+        <v>92</v>
       </c>
       <c r="H90" s="2">
-        <v>95</v>
+        <v>87</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A91" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="B91" s="2">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C91" s="2">
         <v>92</v>
@@ -3191,91 +3191,91 @@
         <v>89</v>
       </c>
       <c r="E91" s="2">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="F91" s="2">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="G91" s="2">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="H91" s="2">
-        <v>82</v>
+        <v>94</v>
       </c>
     </row>
     <row r="92" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A92" t="s">
+        <v>105</v>
+      </c>
+      <c r="B92" s="2">
+        <v>74</v>
+      </c>
+      <c r="C92" s="2">
+        <v>90</v>
+      </c>
+      <c r="D92" s="2">
+        <v>87</v>
+      </c>
+      <c r="E92" s="2">
+        <v>82</v>
+      </c>
+      <c r="F92" s="2">
         <v>98</v>
       </c>
-      <c r="B92" s="2">
-        <v>84</v>
-      </c>
-      <c r="C92" s="2">
-        <v>86</v>
-      </c>
-      <c r="D92" s="2">
+      <c r="G92" s="2">
         <v>90</v>
       </c>
-      <c r="E92" s="2">
-        <v>92</v>
-      </c>
-      <c r="F92" s="2">
-        <v>99</v>
-      </c>
-      <c r="G92" s="2">
-        <v>84</v>
-      </c>
       <c r="H92" s="2">
-        <v>77</v>
+        <v>96</v>
       </c>
     </row>
     <row r="93" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A93" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="B93" s="2">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="C93" s="2">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D93" s="2">
+        <v>93</v>
+      </c>
+      <c r="E93" s="2">
         <v>88</v>
-      </c>
-      <c r="E93" s="2">
-        <v>90</v>
       </c>
       <c r="F93" s="2">
         <v>90</v>
       </c>
       <c r="G93" s="2">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="H93" s="2">
-        <v>86</v>
+        <v>94</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A94" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="B94" s="2">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C94" s="2">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D94" s="2">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="E94" s="2">
         <v>94</v>
       </c>
       <c r="F94" s="2">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="G94" s="2">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="H94" s="2">
         <v>85</v>
@@ -3283,1177 +3283,995 @@
     </row>
     <row r="95" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A95" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B95" s="2">
+        <v>96</v>
+      </c>
+      <c r="C95" s="2">
+        <v>96</v>
+      </c>
+      <c r="D95" s="2">
+        <v>98</v>
+      </c>
+      <c r="E95" s="2">
+        <v>91</v>
+      </c>
+      <c r="F95" s="2">
+        <v>85</v>
+      </c>
+      <c r="G95" s="2">
         <v>83</v>
       </c>
-      <c r="C95" s="2">
-        <v>93</v>
-      </c>
-      <c r="D95" s="2">
-        <v>80</v>
-      </c>
-      <c r="E95" s="2">
-        <v>84</v>
-      </c>
-      <c r="F95" s="2">
-        <v>82</v>
-      </c>
-      <c r="G95" s="2">
-        <v>96</v>
-      </c>
       <c r="H95" s="2">
-        <v>98</v>
+        <v>76</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A96" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="B96" s="2">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="C96" s="2">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D96" s="2">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="E96" s="2">
         <v>84</v>
       </c>
       <c r="F96" s="2">
+        <v>72</v>
+      </c>
+      <c r="G96" s="2">
+        <v>92</v>
+      </c>
+      <c r="H96" s="2">
         <v>80</v>
-      </c>
-      <c r="G96" s="2">
-        <v>99</v>
-      </c>
-      <c r="H96" s="2">
-        <v>89</v>
       </c>
     </row>
     <row r="97" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A97" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="B97" s="2">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C97" s="2">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="D97" s="2">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E97" s="2">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="F97" s="2">
-        <v>86</v>
+        <v>99</v>
       </c>
       <c r="G97" s="2">
-        <v>92</v>
+        <v>76</v>
       </c>
       <c r="H97" s="2">
-        <v>87</v>
+        <v>94</v>
       </c>
     </row>
     <row r="98" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A98" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B98" s="2">
-        <v>91</v>
+        <v>82</v>
       </c>
       <c r="C98" s="2">
+        <v>87</v>
+      </c>
+      <c r="D98" s="2">
         <v>92</v>
       </c>
-      <c r="D98" s="2">
-        <v>89</v>
-      </c>
       <c r="E98" s="2">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F98" s="2">
         <v>89</v>
       </c>
       <c r="G98" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="H98" s="2">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A99" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="B99" s="2">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="C99" s="2">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="D99" s="2">
+        <v>89</v>
+      </c>
+      <c r="E99" s="2">
+        <v>95</v>
+      </c>
+      <c r="F99" s="2">
+        <v>95</v>
+      </c>
+      <c r="G99" s="2">
+        <v>89</v>
+      </c>
+      <c r="H99" s="2">
         <v>87</v>
-      </c>
-      <c r="E99" s="2">
-        <v>82</v>
-      </c>
-      <c r="F99" s="2">
-        <v>98</v>
-      </c>
-      <c r="G99" s="2">
-        <v>90</v>
-      </c>
-      <c r="H99" s="2">
-        <v>96</v>
       </c>
     </row>
     <row r="100" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A100" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="B100" s="2">
-        <v>95</v>
+        <v>74</v>
       </c>
       <c r="C100" s="2">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="D100" s="2">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="E100" s="2">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="F100" s="2">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="G100" s="2">
-        <v>74</v>
+        <v>96</v>
       </c>
       <c r="H100" s="2">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A101" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B101" s="2">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="C101" s="2">
+        <v>85</v>
+      </c>
+      <c r="D101" s="2">
+        <v>86</v>
+      </c>
+      <c r="E101" s="2">
+        <v>84</v>
+      </c>
+      <c r="F101" s="2">
+        <v>83</v>
+      </c>
+      <c r="G101" s="2">
         <v>92</v>
       </c>
-      <c r="D101" s="2">
-        <v>92</v>
-      </c>
-      <c r="E101" s="2">
-        <v>94</v>
-      </c>
-      <c r="F101" s="2">
-        <v>89</v>
-      </c>
-      <c r="G101" s="2">
-        <v>88</v>
-      </c>
       <c r="H101" s="2">
-        <v>85</v>
+        <v>98</v>
       </c>
     </row>
     <row r="102" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A102" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="B102" s="2">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C102" s="2">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D102" s="2">
+        <v>94</v>
+      </c>
+      <c r="E102" s="2">
+        <v>86</v>
+      </c>
+      <c r="F102" s="2">
+        <v>80</v>
+      </c>
+      <c r="G102" s="2">
+        <v>92</v>
+      </c>
+      <c r="H102" s="2">
         <v>98</v>
-      </c>
-      <c r="E102" s="2">
-        <v>91</v>
-      </c>
-      <c r="F102" s="2">
-        <v>85</v>
-      </c>
-      <c r="G102" s="2">
-        <v>83</v>
-      </c>
-      <c r="H102" s="2">
-        <v>76</v>
       </c>
     </row>
     <row r="103" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A103" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="B103" s="2">
-        <v>96</v>
+        <v>74</v>
       </c>
       <c r="C103" s="2">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="D103" s="2">
-        <v>99</v>
+        <v>95</v>
       </c>
       <c r="E103" s="2">
+        <v>91</v>
+      </c>
+      <c r="F103" s="2">
+        <v>91</v>
+      </c>
+      <c r="G103" s="2">
         <v>84</v>
       </c>
-      <c r="F103" s="2">
-        <v>72</v>
-      </c>
-      <c r="G103" s="2">
-        <v>92</v>
-      </c>
       <c r="H103" s="2">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="104" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A104" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B104" s="2">
+        <v>95</v>
+      </c>
+      <c r="C104" s="2">
+        <v>96</v>
+      </c>
+      <c r="D104" s="2">
+        <v>91</v>
+      </c>
+      <c r="E104" s="2">
         <v>88</v>
       </c>
-      <c r="C104" s="2">
-        <v>94</v>
-      </c>
-      <c r="D104" s="2">
-        <v>94</v>
-      </c>
-      <c r="E104" s="2">
-        <v>100</v>
-      </c>
       <c r="F104" s="2">
+        <v>74</v>
+      </c>
+      <c r="G104" s="2">
         <v>99</v>
       </c>
-      <c r="G104" s="2">
-        <v>76</v>
-      </c>
       <c r="H104" s="2">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
     <row r="105" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A105" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="B105" s="2">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C105" s="2">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D105" s="2">
         <v>92</v>
       </c>
       <c r="E105" s="2">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="F105" s="2">
         <v>89</v>
       </c>
       <c r="G105" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="H105" s="2">
-        <v>96</v>
+        <v>82</v>
       </c>
     </row>
     <row r="106" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A106" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="B106" s="2">
-        <v>86</v>
+        <v>65</v>
       </c>
       <c r="C106" s="2">
-        <v>95</v>
+        <v>77</v>
       </c>
       <c r="D106" s="2">
         <v>89</v>
       </c>
       <c r="E106" s="2">
-        <v>95</v>
+        <v>76</v>
       </c>
       <c r="F106" s="2">
-        <v>95</v>
+        <v>60</v>
       </c>
       <c r="G106" s="2">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="H106" s="2">
-        <v>87</v>
+        <v>76</v>
       </c>
     </row>
     <row r="107" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A107" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B107" s="2">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C107" s="2">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D107" s="2">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E107" s="2">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="F107" s="2">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="G107" s="2">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="H107" s="2">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="108" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A108" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="B108" s="2">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="C108" s="2">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D108" s="2">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="E108" s="2">
+        <v>91</v>
+      </c>
+      <c r="F108" s="2">
+        <v>88</v>
+      </c>
+      <c r="G108" s="2">
+        <v>79</v>
+      </c>
+      <c r="H108" s="2">
         <v>84</v>
-      </c>
-      <c r="F108" s="2">
-        <v>83</v>
-      </c>
-      <c r="G108" s="2">
-        <v>92</v>
-      </c>
-      <c r="H108" s="2">
-        <v>98</v>
       </c>
     </row>
     <row r="109" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A109" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="B109" s="2">
-        <v>90</v>
+        <v>81</v>
       </c>
       <c r="C109" s="2">
+        <v>89</v>
+      </c>
+      <c r="D109" s="2">
+        <v>70</v>
+      </c>
+      <c r="E109" s="2">
+        <v>77</v>
+      </c>
+      <c r="F109" s="2">
+        <v>78</v>
+      </c>
+      <c r="G109" s="2">
         <v>93</v>
       </c>
-      <c r="D109" s="2">
-        <v>94</v>
-      </c>
-      <c r="E109" s="2">
-        <v>86</v>
-      </c>
-      <c r="F109" s="2">
-        <v>80</v>
-      </c>
-      <c r="G109" s="2">
-        <v>92</v>
-      </c>
       <c r="H109" s="2">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="110" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A110" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="B110" s="2">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="C110" s="2">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D110" s="2">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="E110" s="2">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="F110" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="G110" s="2">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="H110" s="2">
-        <v>79</v>
+        <v>76</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A111" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="B111" s="2">
+        <v>74</v>
+      </c>
+      <c r="C111" s="2">
+        <v>88</v>
+      </c>
+      <c r="D111" s="2">
+        <v>96</v>
+      </c>
+      <c r="E111" s="2">
+        <v>90</v>
+      </c>
+      <c r="F111" s="2">
+        <v>86</v>
+      </c>
+      <c r="G111" s="2">
         <v>95</v>
       </c>
-      <c r="C111" s="2">
-        <v>96</v>
-      </c>
-      <c r="D111" s="2">
-        <v>91</v>
-      </c>
-      <c r="E111" s="2">
-        <v>88</v>
-      </c>
-      <c r="F111" s="2">
-        <v>74</v>
-      </c>
-      <c r="G111" s="2">
-        <v>99</v>
-      </c>
       <c r="H111" s="2">
-        <v>92</v>
+        <v>89</v>
       </c>
     </row>
     <row r="112" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A112" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="B112" s="2">
+        <v>89</v>
+      </c>
+      <c r="C112" s="2">
         <v>87</v>
       </c>
-      <c r="C112" s="2">
-        <v>94</v>
-      </c>
       <c r="D112" s="2">
+        <v>96</v>
+      </c>
+      <c r="E112" s="2">
         <v>92</v>
-      </c>
-      <c r="E112" s="2">
-        <v>94</v>
       </c>
       <c r="F112" s="2">
         <v>89</v>
       </c>
       <c r="G112" s="2">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H112" s="2">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="113" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A113" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="B113" s="2">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="C113" s="2">
-        <v>77</v>
+        <v>97</v>
       </c>
       <c r="D113" s="2">
-        <v>89</v>
+        <v>78</v>
       </c>
       <c r="E113" s="2">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="F113" s="2">
-        <v>60</v>
+        <v>81</v>
       </c>
       <c r="G113" s="2">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="H113" s="2">
-        <v>76</v>
+        <v>98</v>
       </c>
     </row>
     <row r="114" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A114" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B114" s="2">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="C114" s="2">
+        <v>86</v>
+      </c>
+      <c r="D114" s="2">
         <v>94</v>
-      </c>
-      <c r="D114" s="2">
-        <v>84</v>
       </c>
       <c r="E114" s="2">
         <v>90</v>
       </c>
       <c r="F114" s="2">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="G114" s="2">
+        <v>76</v>
+      </c>
+      <c r="H114" s="2">
         <v>79</v>
-      </c>
-      <c r="H114" s="2">
-        <v>91</v>
       </c>
     </row>
     <row r="115" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A115" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="B115" s="2">
+        <v>87</v>
+      </c>
+      <c r="C115" s="2">
         <v>83</v>
       </c>
-      <c r="C115" s="2">
-        <v>89</v>
-      </c>
       <c r="D115" s="2">
+        <v>86</v>
+      </c>
+      <c r="E115" s="2">
+        <v>78</v>
+      </c>
+      <c r="F115" s="2">
+        <v>74</v>
+      </c>
+      <c r="G115" s="2">
         <v>92</v>
       </c>
-      <c r="E115" s="2">
-        <v>91</v>
-      </c>
-      <c r="F115" s="2">
-        <v>88</v>
-      </c>
-      <c r="G115" s="2">
-        <v>79</v>
-      </c>
       <c r="H115" s="2">
-        <v>84</v>
+        <v>99</v>
       </c>
     </row>
     <row r="116" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A116" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B116" s="2">
-        <v>81</v>
+        <v>91</v>
       </c>
       <c r="C116" s="2">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="D116" s="2">
-        <v>70</v>
+        <v>93</v>
       </c>
       <c r="E116" s="2">
-        <v>77</v>
+        <v>88</v>
       </c>
       <c r="F116" s="2">
-        <v>78</v>
+        <v>94</v>
       </c>
       <c r="G116" s="2">
-        <v>93</v>
+        <v>84</v>
       </c>
       <c r="H116" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
     </row>
     <row r="117" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A117" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B117" s="2">
+        <v>78</v>
+      </c>
+      <c r="C117" s="2">
+        <v>93</v>
+      </c>
+      <c r="D117" s="2">
         <v>88</v>
       </c>
-      <c r="C117" s="2">
-        <v>88</v>
-      </c>
-      <c r="D117" s="2">
-        <v>100</v>
-      </c>
       <c r="E117" s="2">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="F117" s="2">
-        <v>78</v>
+        <v>66</v>
       </c>
       <c r="G117" s="2">
-        <v>82</v>
+        <v>98</v>
       </c>
       <c r="H117" s="2">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="118" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A118" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="B118" s="2">
-        <v>74</v>
+        <v>86</v>
       </c>
       <c r="C118" s="2">
         <v>88</v>
       </c>
       <c r="D118" s="2">
+        <v>95</v>
+      </c>
+      <c r="E118" s="2">
+        <v>94</v>
+      </c>
+      <c r="F118" s="2">
         <v>96</v>
       </c>
-      <c r="E118" s="2">
-        <v>90</v>
-      </c>
-      <c r="F118" s="2">
+      <c r="G118" s="2">
         <v>86</v>
       </c>
-      <c r="G118" s="2">
-        <v>95</v>
-      </c>
       <c r="H118" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A119" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="B119" s="2">
+        <v>78</v>
+      </c>
+      <c r="C119" s="2">
+        <v>88</v>
+      </c>
+      <c r="D119" s="2">
+        <v>98</v>
+      </c>
+      <c r="E119" s="2">
+        <v>88</v>
+      </c>
+      <c r="F119" s="2">
+        <v>82</v>
+      </c>
+      <c r="G119" s="2">
         <v>89</v>
       </c>
-      <c r="C119" s="2">
-        <v>87</v>
-      </c>
-      <c r="D119" s="2">
-        <v>96</v>
-      </c>
-      <c r="E119" s="2">
-        <v>92</v>
-      </c>
-      <c r="F119" s="2">
-        <v>89</v>
-      </c>
-      <c r="G119" s="2">
-        <v>88</v>
-      </c>
       <c r="H119" s="2">
-        <v>79</v>
+        <v>81</v>
       </c>
     </row>
     <row r="120" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A120" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="B120" s="2">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="C120" s="2">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="D120" s="2">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="E120" s="2">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="F120" s="2">
-        <v>81</v>
+        <v>94</v>
       </c>
       <c r="G120" s="2">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="H120" s="2">
-        <v>98</v>
+        <v>91</v>
       </c>
     </row>
     <row r="121" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A121" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="B121" s="2">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C121" s="2">
+        <v>95</v>
+      </c>
+      <c r="D121" s="2">
+        <v>91</v>
+      </c>
+      <c r="E121" s="2">
+        <v>94</v>
+      </c>
+      <c r="F121" s="2">
+        <v>88</v>
+      </c>
+      <c r="G121" s="2">
+        <v>90</v>
+      </c>
+      <c r="H121" s="2">
         <v>86</v>
-      </c>
-      <c r="D121" s="2">
-        <v>94</v>
-      </c>
-      <c r="E121" s="2">
-        <v>90</v>
-      </c>
-      <c r="F121" s="2">
-        <v>87</v>
-      </c>
-      <c r="G121" s="2">
-        <v>76</v>
-      </c>
-      <c r="H121" s="2">
-        <v>79</v>
       </c>
     </row>
     <row r="122" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A122" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="B122" s="2">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C122" s="2">
-        <v>83</v>
+        <v>93</v>
       </c>
       <c r="D122" s="2">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E122" s="2">
-        <v>78</v>
+        <v>92</v>
       </c>
       <c r="F122" s="2">
-        <v>74</v>
+        <v>94</v>
       </c>
       <c r="G122" s="2">
-        <v>92</v>
+        <v>80</v>
       </c>
       <c r="H122" s="2">
-        <v>99</v>
+        <v>84</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A123" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="B123" s="2">
         <v>91</v>
       </c>
       <c r="C123" s="2">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="D123" s="2">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="E123" s="2">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="F123" s="2">
-        <v>94</v>
+        <v>78</v>
       </c>
       <c r="G123" s="2">
-        <v>84</v>
+        <v>97</v>
       </c>
       <c r="H123" s="2">
-        <v>82</v>
+        <v>85</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A124" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="B124" s="2">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="C124" s="2">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="D124" s="2">
-        <v>88</v>
+        <v>98</v>
       </c>
       <c r="E124" s="2">
+        <v>90</v>
+      </c>
+      <c r="F124" s="2">
+        <v>68</v>
+      </c>
+      <c r="G124" s="2">
+        <v>91</v>
+      </c>
+      <c r="H124" s="2">
         <v>84</v>
-      </c>
-      <c r="F124" s="2">
-        <v>66</v>
-      </c>
-      <c r="G124" s="2">
-        <v>98</v>
-      </c>
-      <c r="H124" s="2">
-        <v>80</v>
       </c>
     </row>
     <row r="125" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A125" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B125" s="2">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C125" s="2">
         <v>88</v>
       </c>
       <c r="D125" s="2">
+        <v>91</v>
+      </c>
+      <c r="E125" s="2">
+        <v>90</v>
+      </c>
+      <c r="F125" s="2">
+        <v>94</v>
+      </c>
+      <c r="G125" s="2">
         <v>95</v>
       </c>
-      <c r="E125" s="2">
-        <v>94</v>
-      </c>
-      <c r="F125" s="2">
-        <v>96</v>
-      </c>
-      <c r="G125" s="2">
-        <v>86</v>
-      </c>
       <c r="H125" s="2">
-        <v>79</v>
+        <v>97</v>
       </c>
     </row>
     <row r="126" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A126" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="B126" s="2">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="C126" s="2">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="D126" s="2">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="E126" s="2">
-        <v>88</v>
+        <v>77</v>
       </c>
       <c r="F126" s="2">
-        <v>82</v>
+        <v>60</v>
       </c>
       <c r="G126" s="2">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="H126" s="2">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="127" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A127" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="B127" s="2">
+        <v>83</v>
+      </c>
+      <c r="C127" s="2">
+        <v>92</v>
+      </c>
+      <c r="D127" s="2">
+        <v>96</v>
+      </c>
+      <c r="E127" s="2">
         <v>86</v>
       </c>
-      <c r="C127" s="2">
+      <c r="F127" s="2">
         <v>90</v>
       </c>
-      <c r="D127" s="2">
-        <v>95</v>
-      </c>
-      <c r="E127" s="2">
-        <v>91</v>
-      </c>
-      <c r="F127" s="2">
-        <v>94</v>
-      </c>
       <c r="G127" s="2">
-        <v>88</v>
+        <v>82</v>
       </c>
       <c r="H127" s="2">
-        <v>91</v>
+        <v>83</v>
       </c>
     </row>
     <row r="128" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A128" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="B128" s="2">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C128" s="2">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="D128" s="2">
-        <v>91</v>
+        <v>78</v>
       </c>
       <c r="E128" s="2">
-        <v>94</v>
+        <v>82</v>
       </c>
       <c r="F128" s="2">
-        <v>88</v>
+        <v>68</v>
       </c>
       <c r="G128" s="2">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="H128" s="2">
-        <v>86</v>
+        <v>72</v>
       </c>
     </row>
     <row r="129" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A129" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="B129" s="2">
+        <v>80</v>
+      </c>
+      <c r="C129" s="2">
         <v>86</v>
       </c>
-      <c r="C129" s="2">
-        <v>93</v>
-      </c>
       <c r="D129" s="2">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="E129" s="2">
-        <v>92</v>
+        <v>86</v>
       </c>
       <c r="F129" s="2">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="G129" s="2">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="H129" s="2">
-        <v>84</v>
+        <v>70</v>
       </c>
     </row>
     <row r="130" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A130" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="B130" s="2">
-        <v>91</v>
+        <v>75</v>
       </c>
       <c r="C130" s="2">
-        <v>100</v>
+        <v>79</v>
       </c>
       <c r="D130" s="2">
-        <v>72</v>
+        <v>82</v>
       </c>
       <c r="E130" s="2">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="F130" s="2">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="G130" s="2">
-        <v>97</v>
+        <v>70</v>
       </c>
       <c r="H130" s="2">
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A131" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="B131" s="2">
-        <v>95</v>
+        <v>70</v>
       </c>
       <c r="C131" s="2">
-        <v>89</v>
+        <v>79</v>
       </c>
       <c r="D131" s="2">
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="E131" s="2">
-        <v>90</v>
+        <v>65</v>
       </c>
       <c r="F131" s="2">
+        <v>72</v>
+      </c>
+      <c r="G131" s="2">
         <v>68</v>
       </c>
-      <c r="G131" s="2">
-        <v>91</v>
-      </c>
       <c r="H131" s="2">
-        <v>84</v>
+        <v>68</v>
       </c>
     </row>
     <row r="132" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A132" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="B132" s="2">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="C132" s="2">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="D132" s="2">
-        <v>91</v>
+        <v>74</v>
       </c>
       <c r="E132" s="2">
-        <v>90</v>
+        <v>82</v>
       </c>
       <c r="F132" s="2">
-        <v>94</v>
+        <v>79</v>
       </c>
       <c r="G132" s="2">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H132" s="2">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="133" spans="1:8" ht="20.100000000000001" customHeight="1">
-      <c r="A133" t="s">
-        <v>139</v>
-      </c>
-      <c r="B133" s="2">
-        <v>85</v>
-      </c>
-      <c r="C133" s="2">
-        <v>82</v>
-      </c>
-      <c r="D133" s="2">
-        <v>92</v>
-      </c>
-      <c r="E133" s="2">
-        <v>77</v>
-      </c>
-      <c r="F133" s="2">
-        <v>60</v>
-      </c>
-      <c r="G133" s="2">
-        <v>97</v>
-      </c>
-      <c r="H133" s="2">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="134" spans="1:8" ht="20.100000000000001" customHeight="1">
-      <c r="A134" t="s">
-        <v>140</v>
-      </c>
-      <c r="B134" s="2">
-        <v>83</v>
-      </c>
-      <c r="C134" s="2">
-        <v>92</v>
-      </c>
-      <c r="D134" s="2">
-        <v>96</v>
-      </c>
-      <c r="E134" s="2">
-        <v>86</v>
-      </c>
-      <c r="F134" s="2">
-        <v>90</v>
-      </c>
-      <c r="G134" s="2">
-        <v>82</v>
-      </c>
-      <c r="H134" s="2">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="135" spans="1:8" ht="20.100000000000001" customHeight="1">
-      <c r="A135" t="s">
-        <v>141</v>
-      </c>
-      <c r="B135" s="2">
-        <v>89</v>
-      </c>
-      <c r="C135" s="2">
-        <v>97</v>
-      </c>
-      <c r="D135" s="2">
-        <v>78</v>
-      </c>
-      <c r="E135" s="2">
-        <v>82</v>
-      </c>
-      <c r="F135" s="2">
-        <v>68</v>
-      </c>
-      <c r="G135" s="2">
-        <v>96</v>
-      </c>
-      <c r="H135" s="2">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="136" spans="1:8" ht="20.100000000000001" customHeight="1">
-      <c r="A136" t="s">
-        <v>142</v>
-      </c>
-      <c r="B136" s="2">
-        <v>80</v>
-      </c>
-      <c r="C136" s="2">
-        <v>86</v>
-      </c>
-      <c r="D136" s="2">
-        <v>86</v>
-      </c>
-      <c r="E136" s="2">
-        <v>86</v>
-      </c>
-      <c r="F136" s="2">
-        <v>100</v>
-      </c>
-      <c r="G136" s="2">
-        <v>68</v>
-      </c>
-      <c r="H136" s="2">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="137" spans="1:8" ht="20.100000000000001" customHeight="1">
-      <c r="A137" t="s">
-        <v>143</v>
-      </c>
-      <c r="B137" s="2">
-        <v>75</v>
-      </c>
-      <c r="C137" s="2">
-        <v>79</v>
-      </c>
-      <c r="D137" s="2">
-        <v>82</v>
-      </c>
-      <c r="E137" s="2">
-        <v>76</v>
-      </c>
-      <c r="F137" s="2">
-        <v>95</v>
-      </c>
-      <c r="G137" s="2">
-        <v>70</v>
-      </c>
-      <c r="H137" s="2">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="138" spans="1:8" ht="20.100000000000001" customHeight="1">
-      <c r="A138" t="s">
-        <v>144</v>
-      </c>
-      <c r="B138" s="2">
-        <v>70</v>
-      </c>
-      <c r="C138" s="2">
-        <v>79</v>
-      </c>
-      <c r="D138" s="2">
-        <v>65</v>
-      </c>
-      <c r="E138" s="2">
-        <v>65</v>
-      </c>
-      <c r="F138" s="2">
-        <v>72</v>
-      </c>
-      <c r="G138" s="2">
-        <v>68</v>
-      </c>
-      <c r="H138" s="2">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="139" spans="1:8" ht="20.100000000000001" customHeight="1">
-      <c r="A139" t="s">
-        <v>145</v>
-      </c>
-      <c r="B139" s="2">
-        <v>93</v>
-      </c>
-      <c r="C139" s="2">
-        <v>100</v>
-      </c>
-      <c r="D139" s="2">
-        <v>74</v>
-      </c>
-      <c r="E139" s="2">
-        <v>82</v>
-      </c>
-      <c r="F139" s="2">
-        <v>79</v>
-      </c>
-      <c r="G139" s="2">
-        <v>96</v>
-      </c>
-      <c r="H139" s="2">
         <v>84</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B139">
-    <cfRule type="colorScale" priority="1">
+  <conditionalFormatting sqref="B2:B132">
+    <cfRule type="colorScale" priority="86">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4464,8 +4282,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C139">
-    <cfRule type="colorScale" priority="2">
+  <conditionalFormatting sqref="C2:C132">
+    <cfRule type="colorScale" priority="88">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4476,8 +4294,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D139">
-    <cfRule type="colorScale" priority="3">
+  <conditionalFormatting sqref="D2:D132">
+    <cfRule type="colorScale" priority="90">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4488,8 +4306,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E139">
-    <cfRule type="colorScale" priority="4">
+  <conditionalFormatting sqref="E2:E132">
+    <cfRule type="colorScale" priority="92">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4500,8 +4318,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F139">
-    <cfRule type="colorScale" priority="5">
+  <conditionalFormatting sqref="F2:F132">
+    <cfRule type="colorScale" priority="94">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4512,8 +4330,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G2:G139">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="G2:G132">
+    <cfRule type="colorScale" priority="96">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -4524,8 +4342,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H139">
-    <cfRule type="colorScale" priority="7">
+  <conditionalFormatting sqref="H2:H132">
+    <cfRule type="colorScale" priority="98">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>

</xml_diff>

<commit_message>
"Win condition updates and padding to reroll"
</commit_message>
<xml_diff>
--- a/site/statindexs/Ratings.xlsx
+++ b/site/statindexs/Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nathaniel\Documents\GitHub\ppro\site\statindexs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22946800-11B3-4135-828C-C11BE574AE36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E09590-43BA-4BD6-8AAE-D8E59ED0D25D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4245" yWindow="1815" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2098" uniqueCount="165">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2098" uniqueCount="166">
   <si>
     <t>Fighter Name</t>
   </si>
@@ -517,6 +517,9 @@
   </si>
   <si>
     <t>Charles Oliveira</t>
+  </si>
+  <si>
+    <t>Rampage Jackson</t>
   </si>
 </sst>
 </file>
@@ -4037,7 +4040,7 @@
     </row>
     <row r="124" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A124" t="s">
-        <v>137</v>
+        <v>165</v>
       </c>
       <c r="B124" s="2">
         <v>95</v>

</xml_diff>

<commit_message>
"Diego Lopes image fix"
</commit_message>
<xml_diff>
--- a/site/statindexs/Ratings.xlsx
+++ b/site/statindexs/Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nathaniel\Documents\GitHub\ppro\site\statindexs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58E09590-43BA-4BD6-8AAE-D8E59ED0D25D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9814EA-647E-4CC5-AE02-CC7CD574D473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4245" yWindow="1815" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2098" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2098" uniqueCount="167">
   <si>
     <t>Fighter Name</t>
   </si>
@@ -520,6 +520,9 @@
   </si>
   <si>
     <t>Rampage Jackson</t>
+  </si>
+  <si>
+    <t>Diego Lopes</t>
   </si>
 </sst>
 </file>
@@ -920,7 +923,7 @@
     </row>
     <row r="4" spans="1:8" ht="20.100000000000001" customHeight="1">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>166</v>
       </c>
       <c r="B4" s="2">
         <v>96</v>

</xml_diff>

<commit_message>
"Rogan and Nina rolls"
</commit_message>
<xml_diff>
--- a/site/statindexs/Ratings.xlsx
+++ b/site/statindexs/Ratings.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nathaniel\Documents\GitHub\ppro\site\statindexs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB9814EA-647E-4CC5-AE02-CC7CD574D473}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42654A3C-FA89-4040-9AE7-B3A1285B9D52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4245" yWindow="1815" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4202,25 +4202,25 @@
         <v>143</v>
       </c>
       <c r="B130" s="2">
-        <v>75</v>
+        <v>21</v>
       </c>
       <c r="C130" s="2">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="D130" s="2">
-        <v>82</v>
+        <v>20</v>
       </c>
       <c r="E130" s="2">
-        <v>76</v>
+        <v>30</v>
       </c>
       <c r="F130" s="2">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G130" s="2">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="H130" s="2">
-        <v>88</v>
+        <v>12</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="20.100000000000001" customHeight="1">
@@ -4228,25 +4228,25 @@
         <v>144</v>
       </c>
       <c r="B131" s="2">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="C131" s="2">
-        <v>79</v>
+        <v>100</v>
       </c>
       <c r="D131" s="2">
-        <v>65</v>
+        <v>3</v>
       </c>
       <c r="E131" s="2">
-        <v>65</v>
+        <v>16</v>
       </c>
       <c r="F131" s="2">
-        <v>72</v>
+        <v>19</v>
       </c>
       <c r="G131" s="2">
-        <v>68</v>
+        <v>30</v>
       </c>
       <c r="H131" s="2">
-        <v>68</v>
+        <v>15</v>
       </c>
     </row>
     <row r="132" spans="1:8" ht="20.100000000000001" customHeight="1">

</xml_diff>